<commit_message>
progress: 44 village workbooks (rw-rtx-3070 2026-10-09T23:40:00Z)
</commit_message>
<xml_diff>
--- a/out/Village_map_of_Tiruvallur_Gummidipoondi_Melpakkam_13.447249_80.074836.xlsx
+++ b/out/Village_map_of_Tiruvallur_Gummidipoondi_Melpakkam_13.447249_80.074836.xlsx
@@ -1214,6 +1214,11 @@
           <t>290</t>
         </is>
       </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -1221,6 +1226,11 @@
           <t>291</t>
         </is>
       </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>1, 10, 11A, 11B, 11C, 11D, 11E, 12, 2, 3, 4, 5, 6, 7A, 7B, 7C, 7D, 7E, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -1228,6 +1238,11 @@
           <t>292</t>
         </is>
       </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>10A, 10B, 11A1, 11A2, 11A3, 11B1, 11B2, 1A1, 1A2A, 1A2B, 1B1, 1B10A, 1B10B, 1B11, 1B12, 1B2, 1B3A, 1B3B, 1B4, 1B5, 1B6, 1B7, 1B8, 1B9, 1C1, 1C2, 1C3, 1C4A, 1C4B, 2A, 2B, 2C, 2D, 2E, 2F, 2G, 2H, 2I, 2J, 3A, 3B, 4A, 4B, 4C, 5A, 5B, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -1235,6 +1250,11 @@
           <t>293</t>
         </is>
       </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>10, 11, 12, 13, 14, 15A, 15B, 16A, 16B, 16C, 17A, 17B, 17C, 17D, 17E, 17F, 18, 19, 1A, 1B, 20, 21, 22, 23, 24, 25, 26, 27A, 27B, 28, 29A, 29B, 2A, 2B, 30, 31, 32, 33, 34A, 34B, 34C, 3A, 3B, 4A, 4B, 4C, 4D1, 4D2, 4D3, 4E1, 4E2, 4F, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -1242,6 +1262,11 @@
           <t>294</t>
         </is>
       </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>10, 11A, 11B, 12, 13, 14, 15, 16, 17, 18, 19, 1A, 1B, 20, 21, 22, 2A, 2B, 2C, 3A, 3B, 3C, 3D, 4A, 4B, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -1249,6 +1274,11 @@
           <t>295</t>
         </is>
       </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 2A, 2B, 2C, 2D, 2E, 3A, 3B, 4A, 4B, 5A, 5B, 6A, 6B, 7, 8A, 8B1, 8B2, 8B3, 8B4, 9A, 9B, 9C, 9D, 9E</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -1256,6 +1286,11 @@
           <t>296</t>
         </is>
       </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 2, 20, 21, 22, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -1263,6 +1298,11 @@
           <t>297</t>
         </is>
       </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 14, 15, 16, 17, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -1270,6 +1310,11 @@
           <t>298</t>
         </is>
       </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -1277,6 +1322,11 @@
           <t>299</t>
         </is>
       </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -1284,6 +1334,11 @@
           <t>300</t>
         </is>
       </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 14, 15, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -1291,6 +1346,11 @@
           <t>301</t>
         </is>
       </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4A, 4B, 4C, 5A, 5B, 5C, 6A, 6B, 7A, 7B</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -1298,6 +1358,11 @@
           <t>302</t>
         </is>
       </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>1, 10A, 10B, 11, 2, 3, 4A1, 4A2, 4B1, 4B2, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -1305,6 +1370,11 @@
           <t>303</t>
         </is>
       </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13A, 13B, 13C, 13D, 13E, 14A, 14B, 15, 16, 17, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -1312,6 +1382,11 @@
           <t>304</t>
         </is>
       </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -1319,6 +1394,11 @@
           <t>305</t>
         </is>
       </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 1D, 1E, 1F, 1G, 1H, 2, 3, 4, 5, 6, 7A, 7B</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -1326,6 +1406,11 @@
           <t>306</t>
         </is>
       </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 2, 3, 4, 5A, 5B, 6, 7A, 7B, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -1333,6 +1418,11 @@
           <t>307</t>
         </is>
       </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 1D1, 1D2A, 1D2B, 1E1, 1E2, 2A, 2B, 3A, 3B, 3C, 4A, 4B1, 4B2, 5A, 5B, 6A, 6B, 7A, 7B, 8A, 8B</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -1340,6 +1430,11 @@
           <t>308</t>
         </is>
       </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>1A1, 1A2, 1A3, 1B1, 1B2, 1C1, 1C2, 2A, 2B, 3A, 3B, 3C, 3D, 3E, 4A, 4B</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -1347,6 +1442,11 @@
           <t>309</t>
         </is>
       </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -1354,6 +1454,11 @@
           <t>310</t>
         </is>
       </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -1361,6 +1466,11 @@
           <t>311</t>
         </is>
       </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>10, 11, 12, 13, 14, 15, 16, 1A, 1B, 2, 3A, 3B, 4, 5A, 5B1, 5B10, 5B11, 5B2, 5B3, 5B4, 5B5, 5B6, 5B7, 5B8, 5B9, 5C1, 5C10, 5C11, 5C12, 5C2, 5C3, 5C4, 5C5, 5C6, 5C7, 5C8, 5C9, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -1368,6 +1478,11 @@
           <t>312</t>
         </is>
       </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 2C, 3, 4, 5</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -1375,6 +1490,11 @@
           <t>313</t>
         </is>
       </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>1, 10A, 10B, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -1382,6 +1502,11 @@
           <t>314</t>
         </is>
       </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 14, 15, 16, 17A, 17B, 18, 2A, 2B, 2C, 2D, 3A1A, 3A1B, 3A2, 3B, 4, 5A, 5B, 5C, 5D, 5E, 5F, 5G, 5H, 5I, 5J, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -1389,6 +1514,11 @@
           <t>315</t>
         </is>
       </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12A, 12B, 13, 14, 15, 16, 17, 18, 19, 2, 20, 21, 22, 23, 24, 25, 26, 27, 3, 4A, 4B, 4C, 4D, 5A, 5B, 5C, 6, 7A, 7B, 7C, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -1396,6 +1526,11 @@
           <t>316</t>
         </is>
       </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>10, 11, 12A, 12B, 13A, 13B, 14, 15, 16, 17, 18, 19, 1A, 1B, 1C, 2, 20, 21, 22, 23, 24, 25A1, 25A2, 25A3, 25B, 26, 27, 28, 29, 3, 30, 31, 32, 33, 34, 35, 4A, 4B, 4C, 5, 6, 7, 8A, 8B, 9</t>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -1403,6 +1538,11 @@
           <t>317</t>
         </is>
       </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -1410,6 +1550,11 @@
           <t>318</t>
         </is>
       </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 14, 15, 16, 17, 2, 3, 4, 5A, 5B, 5C, 5D, 5E, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
@@ -1417,6 +1562,11 @@
           <t>319</t>
         </is>
       </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -1424,6 +1574,11 @@
           <t>320</t>
         </is>
       </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 1D, 1E, 2A, 2B, 2C, 3, 4, 5, 6A, 6B, 7, 8</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -1431,6 +1586,11 @@
           <t>321</t>
         </is>
       </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -1438,6 +1598,11 @@
           <t>322</t>
         </is>
       </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 14, 15, 16, 17, 18A, 18B, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
@@ -1445,6 +1610,11 @@
           <t>323</t>
         </is>
       </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -1452,6 +1622,11 @@
           <t>324</t>
         </is>
       </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>10, 11, 12, 13, 1A, 1B, 2A, 2B, 3, 4, 5A, 5B, 6A, 6B, 7A, 7B, 8A, 8B, 8C, 9A, 9B</t>
+        </is>
+      </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
@@ -1459,6 +1634,11 @@
           <t>325</t>
         </is>
       </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
@@ -1466,6 +1646,11 @@
           <t>326</t>
         </is>
       </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
@@ -1473,6 +1658,11 @@
           <t>327</t>
         </is>
       </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
@@ -1480,6 +1670,11 @@
           <t>328</t>
         </is>
       </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4</t>
+        </is>
+      </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
@@ -1487,6 +1682,11 @@
           <t>329</t>
         </is>
       </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
@@ -1494,6 +1694,11 @@
           <t>330</t>
         </is>
       </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
@@ -1501,6 +1706,11 @@
           <t>331</t>
         </is>
       </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
@@ -1508,6 +1718,11 @@
           <t>332</t>
         </is>
       </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
@@ -1515,6 +1730,11 @@
           <t>333</t>
         </is>
       </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4A, 4B, 4C, 4D, 4E, 4F, 4G, 5</t>
+        </is>
+      </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
@@ -1522,6 +1742,11 @@
           <t>334</t>
         </is>
       </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
@@ -1529,6 +1754,11 @@
           <t>335</t>
         </is>
       </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>1, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
@@ -1536,6 +1766,11 @@
           <t>336</t>
         </is>
       </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>1, 2, 3</t>
+        </is>
+      </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
@@ -1543,6 +1778,11 @@
           <t>337</t>
         </is>
       </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
@@ -1550,6 +1790,11 @@
           <t>338</t>
         </is>
       </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
@@ -1557,6 +1802,11 @@
           <t>339</t>
         </is>
       </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
@@ -1564,6 +1814,11 @@
           <t>340</t>
         </is>
       </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
@@ -1571,6 +1826,11 @@
           <t>341</t>
         </is>
       </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
@@ -1578,6 +1838,11 @@
           <t>342</t>
         </is>
       </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>10A, 10B, 11, 12A, 12B, 13, 14, 15, 16, 17A, 17B, 18, 19, 1A, 1B, 1C, 1D, 1E, 1F, 2, 20, 3, 4A, 4B, 4C, 5, 6, 7A, 7B, 7C, 7D, 8A1, 8A2, 8B1, 8B2, 9</t>
+        </is>
+      </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
@@ -1585,6 +1850,11 @@
           <t>343</t>
         </is>
       </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13A, 13B, 13C, 14, 15, 16, 2, 3, 4, 5A, 5B, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
@@ -1592,6 +1862,11 @@
           <t>344</t>
         </is>
       </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 14, 15, 2, 3, 4A, 4B, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
@@ -1599,6 +1874,11 @@
           <t>345</t>
         </is>
       </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B1, 2B2, 2C, 2D, 2E, 2F, 2G, 2H, 2I, 2J, 2K, 3, 4A, 4B, 5</t>
+        </is>
+      </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
@@ -1606,6 +1886,11 @@
           <t>346</t>
         </is>
       </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>1, 10A, 10B, 10C, 11, 12, 13, 14, 15A, 15B, 15C, 15D, 16, 17, 18, 19A1, 19A2, 19B, 2, 20, 21, 22, 3, 4, 5A, 5B, 6A, 6B, 6C, 6D, 6E, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
@@ -1613,6 +1898,11 @@
           <t>347</t>
         </is>
       </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>10A, 10B, 11, 12A, 12B, 13, 14, 15A, 15B, 15C, 15D, 15E, 15F, 15G, 15H, 15I, 15J, 15K, 16, 17, 18A, 18B1, 18B2, 18C, 18D, 1A, 1B, 1C, 1D1, 1D2, 1E, 1F1, 1F2, 1G, 1H, 1I, 1J, 1K, 2A, 2B, 3, 4, 5A, 5B, 6, 7, 8, 9A, 9B</t>
+        </is>
+      </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
@@ -1620,6 +1910,11 @@
           <t>348</t>
         </is>
       </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 1A, 1B, 1C1, 1C2, 1C3, 1D, 1E, 1F, 2, 20, 21, 22, 23, 24, 25, 26, 27, 28, 29, 3, 30, 31, 32, 33, 34, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
@@ -1627,6 +1922,11 @@
           <t>349</t>
         </is>
       </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>1, 10A, 10B, 11, 12, 13, 14, 15, 16, 17, 18, 19A, 19B, 2, 20, 21, 22, 3, 4, 5A, 5B, 6, 7, 8A, 8B, 8C, 9</t>
+        </is>
+      </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
@@ -1634,6 +1934,11 @@
           <t>350</t>
         </is>
       </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19A, 19B, 2, 20, 21, 22, 23, 24, 25, 26, 27, 28, 29, 3, 30, 31, 32, 33, 35, 4, 5, 6, 7, 8A, 8B, 8C, 9</t>
+        </is>
+      </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
@@ -1641,6 +1946,11 @@
           <t>351</t>
         </is>
       </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13A, 13B, 13C, 13D, 14, 15, 16, 2, 3, 4, 5A, 5B, 5C, 6, 7, 8A, 8B, 9</t>
+        </is>
+      </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
@@ -1648,6 +1958,11 @@
           <t>352</t>
         </is>
       </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>1, 10A, 10B, 11A, 11B, 12A, 12B, 12C, 12D, 12E, 12F, 12G, 13, 14A, 14B, 14C, 15, 16, 17, 18A, 18B, 18C, 18D, 19A, 19B, 20, 21, 22, 23, 24, 25, 26, 27, 28, 29, 2A1, 2A2, 2B, 3, 30, 31, 32, 33, 34, 35A, 35B, 36, 37, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
@@ -1655,6 +1970,11 @@
           <t>353</t>
         </is>
       </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 14A, 14B, 15, 16, 17, 18A, 18B, 19, 2, 20, 21, 22, 23, 24, 25, 26, 27, 28, 29, 3, 30, 31, 32, 33, 34, 4, 5, 6A, 6B, 7A, 7B, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
@@ -1662,6 +1982,11 @@
           <t>354</t>
         </is>
       </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 14, 15A, 15B, 15C, 15D, 16A, 16B, 16C, 16D1, 16D2, 16E, 16F, 16G, 16H, 17, 18, 19A, 19B, 19C, 19D, 2, 20, 21, 22, 23A, 23B, 23C, 3, 4, 5, 6A, 6B, 7, 8A, 8B, 8C, 9A, 9B, 9C1, 9C2, 9D, 9E</t>
+        </is>
+      </c>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
@@ -1669,6 +1994,11 @@
           <t>355</t>
         </is>
       </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 2, 3A, 3B, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
@@ -1676,6 +2006,11 @@
           <t>356</t>
         </is>
       </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>1, 10A, 10B, 11, 12, 13, 14, 15, 16, 17, 18, 19, 2, 20, 21, 22, 23, 24, 25A, 25B, 26, 27, 28, 29, 3, 30, 4, 5, 6, 7, 8, 9A, 9B</t>
+        </is>
+      </c>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
@@ -1683,6 +2018,11 @@
           <t>357</t>
         </is>
       </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 2, 20, 21, 22, 23, 24, 25, 26, 27, 28, 29, 3, 30, 31, 32, 33, 34, 35, 4, 5, 6A, 6B, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
@@ -1690,6 +2030,11 @@
           <t>358</t>
         </is>
       </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>1, 10, 11A, 11B, 12, 13, 14, 15, 2, 3, 4, 5A, 5B, 5C, 6A, 6B, 6C, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
@@ -1697,6 +2042,11 @@
           <t>359</t>
         </is>
       </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 2, 20, 21A, 21B, 21C, 22, 23, 24, 25, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
@@ -1704,6 +2054,11 @@
           <t>360</t>
         </is>
       </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 14, 15, 16, 17A1, 17A2, 17B, 18, 2, 3, 4, 5, 6, 7, 8A, 8B, 9</t>
+        </is>
+      </c>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
@@ -1711,6 +2066,11 @@
           <t>361</t>
         </is>
       </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5, 6</t>
+        </is>
+      </c>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
@@ -1718,6 +2078,11 @@
           <t>362</t>
         </is>
       </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
@@ -1725,6 +2090,11 @@
           <t>363</t>
         </is>
       </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5</t>
+        </is>
+      </c>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
@@ -1732,6 +2102,11 @@
           <t>364</t>
         </is>
       </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12A, 12B, 12C, 12D, 12E, 13, 14A, 14B, 14C, 15, 16, 2, 3, 4, 5A, 5B, 5C, 6, 7, 8, 9A, 9B</t>
+        </is>
+      </c>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
@@ -1739,6 +2114,11 @@
           <t>365</t>
         </is>
       </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12A1, 12A2, 12A3, 12B, 12C1, 12C2, 12C3, 12D, 12E, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23, 24, 2A, 2B, 3, 4, 5, 6A1, 6A2, 6A3, 6B, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
@@ -1746,6 +2126,11 @@
           <t>366</t>
         </is>
       </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>1, 10A, 10B, 11, 12A, 12B, 13, 14A, 14B, 15A, 15B, 16A, 16B, 16C, 16D1, 16D2, 17A, 17B, 17C, 18, 19, 2, 20, 3A, 3B, 4A, 4B, 4C, 4D, 4E, 4F, 4G, 5, 6A, 6B, 7, 8, 9A1, 9A2, 9B, 9C, 9D, 9E, 9F</t>
+        </is>
+      </c>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
@@ -1753,6 +2138,11 @@
           <t>367</t>
         </is>
       </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>1A, 1B, 2A, 2B, 2C, 3, 4, 5A, 5B, 6A, 6B1A1, 6B1A2, 6B1B, 6B2, 6C1, 6C2, 6C3, 6D, 6E1, 6E2, 6F1, 6F2, 6F3, 6F4, 6F5, 6G, 7A, 7B, 7C1, 7C2, 7D</t>
+        </is>
+      </c>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
@@ -1760,6 +2150,11 @@
           <t>368</t>
         </is>
       </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 1D, 1E1, 1E2, 1E3, 2A, 2B, 2C1, 2C2, 2D1, 2D2, 3A, 3B1, 3B2, 4A1, 4A2, 4B, 4C1, 4C2, 4D, 4E1A1, 4E1A2, 4E1B, 4E2</t>
+        </is>
+      </c>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
@@ -1767,6 +2162,11 @@
           <t>369</t>
         </is>
       </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B1, 2B2, 2C1, 2C2, 3A, 3B, 4, 5A, 5B, 6A, 6B, 7A, 7B, 7C</t>
+        </is>
+      </c>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
@@ -1774,6 +2174,11 @@
           <t>370</t>
         </is>
       </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>1, 2A, 2B, 2C, 3A1, 3A2, 3A3, 3A4, 3A5, 3A6, 3B, 4A, 4B, 5A, 5B, 5C, 5D, 5E, 6A1, 6A2, 6B, 7A1, 7A2, 7B1, 7B2, 8A, 8B</t>
+        </is>
+      </c>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
@@ -1781,6 +2186,11 @@
           <t>371</t>
         </is>
       </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 2, 3A, 3B, 3C, 4, 5, 6A1A1, 6A1A2, 6A1B, 6A2, 6B, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
@@ -1788,6 +2198,11 @@
           <t>372</t>
         </is>
       </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>10A1, 10A2, 10B, 11, 12, 13, 14, 15, 16, 1A, 1B, 2, 3, 4, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
@@ -1795,6 +2210,11 @@
           <t>373</t>
         </is>
       </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5</t>
+        </is>
+      </c>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
@@ -1802,6 +2222,11 @@
           <t>374</t>
         </is>
       </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 14, 15A, 15B, 16, 17, 18, 2A, 2B, 3, 4A, 4B, 5, 6, 7, 8, 9</t>
+        </is>
+      </c>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
@@ -1809,6 +2234,11 @@
           <t>375</t>
         </is>
       </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 2, 20, 3, 4, 5, 6, 7, 8, 9A, 9B1, 9B2</t>
+        </is>
+      </c>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
@@ -1816,6 +2246,11 @@
           <t>376</t>
         </is>
       </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>1A, 1B, 1C, 2</t>
+        </is>
+      </c>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
@@ -1823,11 +2258,21 @@
           <t>377</t>
         </is>
       </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>1, 2, 3, 4, 5, 6</t>
+        </is>
+      </c>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
           <t>378</t>
+        </is>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>1, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 22A, 22B, 23, 24, 25, 2A, 2B, 3A, 3B, 3C, 3D, 3E, 4, 5A, 5B, 6, 7, 8A, 8B, 9</t>
         </is>
       </c>
     </row>

</xml_diff>